<commit_message>
better fix for exec
</commit_message>
<xml_diff>
--- a/company_data.xlsx
+++ b/company_data.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1044,6 +1044,44 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>S-9009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sunny Imaging center</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1144,12 +1182,12 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-04-21 00:00:00</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-07-17 00:00:00</t>
+          <t>2027-01-29</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1157,7 +1195,11 @@
           <t>Alvarez</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Kaggwa</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1590,7 +1632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1636,15 +1678,10 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>date_done</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>date_completed</t>
         </is>
@@ -1693,15 +1730,14 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Monitor screen was replaced</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>2026-07-15 03:00:51.851000</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Monitor screen was replaced</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1746,15 +1782,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Valve bearings were replaced</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>2026-07-15 03:03:07.032000</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Valve bearings were replaced</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1797,15 +1832,58 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Client needs to add padding when keeping the item in storage.</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Client needs to add padding when keeping the item in storage.</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
           <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R-1004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>M-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Infusion Pump A200</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sunny Imaging center</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">testing </t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Kaggwa</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>

</xml_diff>